<commit_message>
Added links to TBA, FRC and Statbotics from Teams tab.
</commit_message>
<xml_diff>
--- a/The Blue Alliance/Templates/scouting_template.xlsx
+++ b/The Blue Alliance/Templates/scouting_template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/johnhurrell/Development/fairport-robotics/ScoutingPASSSync/The Blue Alliance/Templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{292C1BDA-8568-D24C-8936-48175E478456}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1233944-BFF3-7F4C-BCD2-A35525035DA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="MatchScoutingData" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">MatchScoutingData!$A$1:$AB$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Team Scores'!$A$2:$Z$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Team Summary'!$A$2:$AE$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Teams!$A$1:$E$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Teams!$A$1:$F$1</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="80">
   <si>
     <t>Key</t>
   </si>
@@ -84,9 +84,6 @@
   </si>
   <si>
     <t>School</t>
-  </si>
-  <si>
-    <t>Rookie Year</t>
   </si>
   <si>
     <t>Start Time</t>
@@ -279,6 +276,15 @@
   </si>
   <si>
     <t>Wrong team was scouted</t>
+  </si>
+  <si>
+    <t>TBA</t>
+  </si>
+  <si>
+    <t>FRC</t>
+  </si>
+  <si>
+    <t>Statbotics</t>
   </si>
 </sst>
 </file>
@@ -507,7 +513,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -559,11 +565,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" textRotation="90"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -583,14 +592,14 @@
     <xf numFmtId="0" fontId="1" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" textRotation="90"/>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" textRotation="90"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -919,7 +928,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C1" s="10" t="s">
         <v>1</v>
@@ -931,73 +940,73 @@
         <v>3</v>
       </c>
       <c r="F1" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="G1" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="G1" s="10" t="s">
+      <c r="H1" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="H1" s="10" t="s">
+      <c r="I1" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="I1" s="10" t="s">
+      <c r="J1" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="J1" s="10" t="s">
+      <c r="K1" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="K1" s="10" t="s">
+      <c r="L1" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="L1" s="10" t="s">
+      <c r="M1" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="M1" s="10" t="s">
+      <c r="N1" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="N1" s="10" t="s">
+      <c r="O1" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="O1" s="10" t="s">
+      <c r="P1" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="P1" s="10" t="s">
+      <c r="Q1" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="Q1" s="10" t="s">
+      <c r="R1" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="R1" s="10" t="s">
+      <c r="S1" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="S1" s="10" t="s">
+      <c r="T1" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="T1" s="10" t="s">
+      <c r="U1" s="10" t="s">
+        <v>60</v>
+      </c>
+      <c r="V1" s="10" t="s">
         <v>34</v>
       </c>
-      <c r="U1" s="10" t="s">
-        <v>61</v>
-      </c>
-      <c r="V1" s="10" t="s">
+      <c r="W1" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="W1" s="10" t="s">
+      <c r="X1" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="X1" s="10" t="s">
+      <c r="Y1" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="Y1" s="10" t="s">
+      <c r="Z1" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="Z1" s="10" t="s">
+      <c r="AA1" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="AA1" s="10" t="s">
+      <c r="AB1" s="10" t="s">
         <v>40</v>
-      </c>
-      <c r="AB1" s="10" t="s">
-        <v>41</v>
       </c>
       <c r="AC1" s="10" t="s">
         <v>4</v>
@@ -20875,17 +20884,16 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:AE32"/>
+  <dimension ref="A1:AC32"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="16.5" customWidth="1"/>
     <col min="2" max="2" width="35" customWidth="1"/>
     <col min="3" max="3" width="50" customWidth="1"/>
-    <col min="4" max="4" width="20" customWidth="1"/>
-    <col min="5" max="5" width="15" customWidth="1"/>
+    <col min="4" max="6" width="12.83203125" style="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:31" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:29" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="5" t="s">
         <v>10</v>
       </c>
@@ -20895,13 +20903,15 @@
       <c r="C1" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="D1" s="5" t="s">
-        <v>13</v>
+      <c r="D1" s="34" t="s">
+        <v>77</v>
       </c>
-      <c r="E1" s="5" t="s">
-        <v>5</v>
+      <c r="E1" s="34" t="s">
+        <v>78</v>
       </c>
-      <c r="F1" s="5"/>
+      <c r="F1" s="34" t="s">
+        <v>79</v>
+      </c>
       <c r="G1" s="5"/>
       <c r="H1" s="5"/>
       <c r="I1" s="5"/>
@@ -20925,52 +20935,50 @@
       <c r="AA1" s="5"/>
       <c r="AB1" s="5"/>
       <c r="AC1" s="5"/>
-      <c r="AD1" s="5"/>
-      <c r="AE1" s="5"/>
-    </row>
-    <row r="2" spans="1:31" ht="16" x14ac:dyDescent="0.2">
+    </row>
+    <row r="2" spans="1:29" ht="16" x14ac:dyDescent="0.2">
       <c r="A2" s="4"/>
     </row>
-    <row r="3" spans="1:31" ht="16" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:29" ht="16" x14ac:dyDescent="0.2">
       <c r="A3" s="4"/>
     </row>
-    <row r="4" spans="1:31" ht="16" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:29" ht="16" x14ac:dyDescent="0.2">
       <c r="A4" s="4"/>
     </row>
-    <row r="5" spans="1:31" ht="16" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:29" ht="16" x14ac:dyDescent="0.2">
       <c r="A5" s="4"/>
     </row>
-    <row r="6" spans="1:31" ht="16" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:29" ht="16" x14ac:dyDescent="0.2">
       <c r="A6" s="4"/>
     </row>
-    <row r="7" spans="1:31" ht="16" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:29" ht="16" x14ac:dyDescent="0.2">
       <c r="A7" s="4"/>
     </row>
-    <row r="8" spans="1:31" ht="16" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:29" ht="16" x14ac:dyDescent="0.2">
       <c r="A8" s="4"/>
     </row>
-    <row r="9" spans="1:31" ht="16" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:29" ht="16" x14ac:dyDescent="0.2">
       <c r="A9" s="4"/>
     </row>
-    <row r="10" spans="1:31" ht="16" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:29" ht="16" x14ac:dyDescent="0.2">
       <c r="A10" s="4"/>
     </row>
-    <row r="11" spans="1:31" ht="16" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:29" ht="16" x14ac:dyDescent="0.2">
       <c r="A11" s="4"/>
     </row>
-    <row r="12" spans="1:31" ht="16" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:29" ht="16" x14ac:dyDescent="0.2">
       <c r="A12" s="4"/>
     </row>
-    <row r="13" spans="1:31" ht="16" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:29" ht="16" x14ac:dyDescent="0.2">
       <c r="A13" s="4"/>
     </row>
-    <row r="14" spans="1:31" ht="16" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:29" ht="16" x14ac:dyDescent="0.2">
       <c r="A14" s="4"/>
     </row>
-    <row r="15" spans="1:31" ht="16" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:29" ht="16" x14ac:dyDescent="0.2">
       <c r="A15" s="4"/>
     </row>
-    <row r="16" spans="1:31" ht="16" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:29" ht="16" x14ac:dyDescent="0.2">
       <c r="A16" s="4"/>
     </row>
     <row r="17" spans="1:1" ht="16" x14ac:dyDescent="0.2">
@@ -21022,7 +21030,7 @@
       <c r="A32" s="4"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E1" xr:uid="{00000000-0009-0000-0000-000002000000}"/>
+  <autoFilter ref="A1:F1" xr:uid="{00000000-0001-0000-0200-000000000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -21043,45 +21051,45 @@
         <v>1</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C1" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="D1" s="7" t="s">
         <v>68</v>
       </c>
-      <c r="D1" s="7" t="s">
+      <c r="E1" s="7" t="s">
         <v>69</v>
       </c>
-      <c r="E1" s="7" t="s">
+      <c r="F1" s="8" t="s">
         <v>70</v>
       </c>
-      <c r="F1" s="8" t="s">
+      <c r="G1" s="8" t="s">
         <v>71</v>
       </c>
-      <c r="G1" s="8" t="s">
+      <c r="H1" s="8" t="s">
         <v>72</v>
       </c>
-      <c r="H1" s="8" t="s">
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="J2" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="J2" t="s">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="J3" s="18" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="J3" s="18" t="s">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="J4" s="20" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="J4" s="20" t="s">
-        <v>76</v>
-      </c>
-    </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.2">
       <c r="J5" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="8" spans="1:10" ht="16" x14ac:dyDescent="0.2">
@@ -21136,117 +21144,117 @@
     <row r="1" spans="1:26" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A1" s="6"/>
       <c r="B1" s="6"/>
-      <c r="C1" s="25" t="s">
+      <c r="C1" s="26" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1" s="27"/>
+      <c r="E1" s="27"/>
+      <c r="F1" s="27"/>
+      <c r="G1" s="27"/>
+      <c r="H1" s="28" t="s">
         <v>15</v>
       </c>
-      <c r="D1" s="26"/>
-      <c r="E1" s="26"/>
-      <c r="F1" s="26"/>
-      <c r="G1" s="26"/>
-      <c r="H1" s="27" t="s">
+      <c r="I1" s="29"/>
+      <c r="J1" s="29"/>
+      <c r="K1" s="29"/>
+      <c r="L1" s="29"/>
+      <c r="M1" s="29"/>
+      <c r="N1" s="29"/>
+      <c r="O1" s="29"/>
+      <c r="P1" s="30" t="s">
         <v>16</v>
       </c>
-      <c r="I1" s="28"/>
-      <c r="J1" s="28"/>
-      <c r="K1" s="28"/>
-      <c r="L1" s="28"/>
-      <c r="M1" s="28"/>
-      <c r="N1" s="28"/>
-      <c r="O1" s="28"/>
-      <c r="P1" s="29" t="s">
-        <v>17</v>
+      <c r="Q1" s="31"/>
+      <c r="R1" s="31"/>
+      <c r="S1" s="31"/>
+      <c r="T1" s="31"/>
+      <c r="U1" s="32" t="s">
+        <v>63</v>
       </c>
-      <c r="Q1" s="30"/>
-      <c r="R1" s="30"/>
-      <c r="S1" s="30"/>
-      <c r="T1" s="30"/>
-      <c r="U1" s="23" t="s">
-        <v>64</v>
-      </c>
-      <c r="V1" s="23"/>
-      <c r="W1" s="23"/>
-      <c r="X1" s="23"/>
-      <c r="Y1" s="23"/>
-      <c r="Z1" s="24"/>
+      <c r="V1" s="32"/>
+      <c r="W1" s="32"/>
+      <c r="X1" s="32"/>
+      <c r="Y1" s="32"/>
+      <c r="Z1" s="33"/>
     </row>
     <row r="2" spans="1:26" ht="130" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
         <v>3</v>
       </c>
       <c r="B2" s="12" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C2" s="13" t="s">
+        <v>41</v>
+      </c>
+      <c r="D2" s="13" t="s">
         <v>42</v>
       </c>
-      <c r="D2" s="13" t="s">
+      <c r="E2" s="13" t="s">
         <v>43</v>
       </c>
-      <c r="E2" s="13" t="s">
+      <c r="F2" s="13" t="s">
         <v>44</v>
       </c>
-      <c r="F2" s="13" t="s">
+      <c r="G2" s="13" t="s">
+        <v>61</v>
+      </c>
+      <c r="H2" s="14" t="s">
+        <v>47</v>
+      </c>
+      <c r="I2" s="14" t="s">
         <v>45</v>
       </c>
-      <c r="G2" s="13" t="s">
-        <v>62</v>
+      <c r="J2" s="14" t="s">
+        <v>46</v>
       </c>
-      <c r="H2" s="14" t="s">
+      <c r="K2" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="I2" s="14" t="s">
-        <v>46</v>
-      </c>
-      <c r="J2" s="14" t="s">
-        <v>47</v>
-      </c>
-      <c r="K2" s="14" t="s">
+      <c r="L2" s="14" t="s">
         <v>49</v>
       </c>
-      <c r="L2" s="14" t="s">
+      <c r="M2" s="14" t="s">
         <v>50</v>
       </c>
-      <c r="M2" s="14" t="s">
+      <c r="N2" s="14" t="s">
         <v>51</v>
       </c>
-      <c r="N2" s="14" t="s">
+      <c r="O2" s="14" t="s">
+        <v>31</v>
+      </c>
+      <c r="P2" s="15" t="s">
         <v>52</v>
       </c>
-      <c r="O2" s="14" t="s">
-        <v>32</v>
-      </c>
-      <c r="P2" s="15" t="s">
+      <c r="Q2" s="15" t="s">
         <v>53</v>
       </c>
-      <c r="Q2" s="15" t="s">
+      <c r="R2" s="15" t="s">
+        <v>60</v>
+      </c>
+      <c r="S2" s="15" t="s">
         <v>54</v>
       </c>
-      <c r="R2" s="15" t="s">
-        <v>61</v>
-      </c>
-      <c r="S2" s="15" t="s">
+      <c r="T2" s="15" t="s">
         <v>55</v>
       </c>
-      <c r="T2" s="15" t="s">
+      <c r="U2" s="21" t="s">
+        <v>64</v>
+      </c>
+      <c r="V2" s="21" t="s">
+        <v>59</v>
+      </c>
+      <c r="W2" s="21" t="s">
         <v>56</v>
       </c>
-      <c r="U2" s="21" t="s">
-        <v>65</v>
-      </c>
-      <c r="V2" s="21" t="s">
-        <v>60</v>
-      </c>
-      <c r="W2" s="21" t="s">
+      <c r="X2" s="21" t="s">
         <v>57</v>
       </c>
-      <c r="X2" s="21" t="s">
+      <c r="Y2" s="21" t="s">
         <v>58</v>
       </c>
-      <c r="Y2" s="21" t="s">
-        <v>59</v>
-      </c>
       <c r="Z2" s="16" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="3" spans="1:26" x14ac:dyDescent="0.2">
@@ -29586,141 +29594,141 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:31" ht="17" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="32" t="s">
+      <c r="A1" s="24" t="s">
         <v>3</v>
       </c>
       <c r="B1" s="6"/>
-      <c r="C1" s="25" t="s">
+      <c r="C1" s="26" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1" s="27"/>
+      <c r="E1" s="27"/>
+      <c r="F1" s="27"/>
+      <c r="G1" s="27"/>
+      <c r="H1" s="28" t="s">
         <v>15</v>
       </c>
-      <c r="D1" s="26"/>
-      <c r="E1" s="26"/>
-      <c r="F1" s="26"/>
-      <c r="G1" s="26"/>
-      <c r="H1" s="27" t="s">
+      <c r="I1" s="29"/>
+      <c r="J1" s="29"/>
+      <c r="K1" s="29"/>
+      <c r="L1" s="29"/>
+      <c r="M1" s="29"/>
+      <c r="N1" s="29"/>
+      <c r="O1" s="29"/>
+      <c r="P1" s="30" t="s">
         <v>16</v>
       </c>
-      <c r="I1" s="28"/>
-      <c r="J1" s="28"/>
-      <c r="K1" s="28"/>
-      <c r="L1" s="28"/>
-      <c r="M1" s="28"/>
-      <c r="N1" s="28"/>
-      <c r="O1" s="28"/>
-      <c r="P1" s="29" t="s">
+      <c r="Q1" s="31"/>
+      <c r="R1" s="31"/>
+      <c r="S1" s="31"/>
+      <c r="T1" s="31"/>
+      <c r="U1" s="32" t="s">
+        <v>63</v>
+      </c>
+      <c r="V1" s="32"/>
+      <c r="W1" s="32"/>
+      <c r="X1" s="32"/>
+      <c r="Y1" s="32"/>
+      <c r="Z1" s="32"/>
+      <c r="AA1" s="23" t="s">
         <v>17</v>
       </c>
-      <c r="Q1" s="30"/>
-      <c r="R1" s="30"/>
-      <c r="S1" s="30"/>
-      <c r="T1" s="30"/>
-      <c r="U1" s="23" t="s">
+      <c r="AB1" s="23"/>
+      <c r="AC1" s="23"/>
+      <c r="AD1" s="23"/>
+      <c r="AE1" s="23"/>
+    </row>
+    <row r="2" spans="1:31" ht="130" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="25"/>
+      <c r="B2" s="12" t="s">
+        <v>65</v>
+      </c>
+      <c r="C2" s="13" t="s">
+        <v>41</v>
+      </c>
+      <c r="D2" s="13" t="s">
+        <v>42</v>
+      </c>
+      <c r="E2" s="13" t="s">
+        <v>43</v>
+      </c>
+      <c r="F2" s="13" t="s">
+        <v>44</v>
+      </c>
+      <c r="G2" s="13" t="s">
+        <v>61</v>
+      </c>
+      <c r="H2" s="14" t="s">
+        <v>47</v>
+      </c>
+      <c r="I2" s="14" t="s">
+        <v>45</v>
+      </c>
+      <c r="J2" s="14" t="s">
+        <v>46</v>
+      </c>
+      <c r="K2" s="14" t="s">
+        <v>48</v>
+      </c>
+      <c r="L2" s="14" t="s">
+        <v>49</v>
+      </c>
+      <c r="M2" s="14" t="s">
+        <v>50</v>
+      </c>
+      <c r="N2" s="14" t="s">
+        <v>51</v>
+      </c>
+      <c r="O2" s="14" t="s">
+        <v>31</v>
+      </c>
+      <c r="P2" s="15" t="s">
+        <v>52</v>
+      </c>
+      <c r="Q2" s="15" t="s">
+        <v>53</v>
+      </c>
+      <c r="R2" s="15" t="s">
+        <v>60</v>
+      </c>
+      <c r="S2" s="15" t="s">
+        <v>54</v>
+      </c>
+      <c r="T2" s="15" t="s">
+        <v>55</v>
+      </c>
+      <c r="U2" s="21" t="s">
         <v>64</v>
       </c>
-      <c r="V1" s="23"/>
-      <c r="W1" s="23"/>
-      <c r="X1" s="23"/>
-      <c r="Y1" s="23"/>
-      <c r="Z1" s="23"/>
-      <c r="AA1" s="31" t="s">
-        <v>18</v>
+      <c r="V2" s="21" t="s">
+        <v>59</v>
       </c>
-      <c r="AB1" s="31"/>
-      <c r="AC1" s="31"/>
-      <c r="AD1" s="31"/>
-      <c r="AE1" s="31"/>
-    </row>
-    <row r="2" spans="1:31" ht="130" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="33"/>
-      <c r="B2" s="12" t="s">
-        <v>66</v>
+      <c r="W2" s="21" t="s">
+        <v>56</v>
       </c>
-      <c r="C2" s="13" t="s">
-        <v>42</v>
+      <c r="X2" s="21" t="s">
+        <v>57</v>
       </c>
-      <c r="D2" s="13" t="s">
-        <v>43</v>
+      <c r="Y2" s="21" t="s">
+        <v>58</v>
       </c>
-      <c r="E2" s="13" t="s">
-        <v>44</v>
-      </c>
-      <c r="F2" s="13" t="s">
-        <v>45</v>
-      </c>
-      <c r="G2" s="13" t="s">
+      <c r="Z2" s="16" t="s">
         <v>62</v>
       </c>
-      <c r="H2" s="14" t="s">
-        <v>48</v>
+      <c r="AA2" s="13" t="s">
+        <v>14</v>
       </c>
-      <c r="I2" s="14" t="s">
-        <v>46</v>
+      <c r="AB2" s="14" t="s">
+        <v>15</v>
       </c>
-      <c r="J2" s="14" t="s">
-        <v>47</v>
+      <c r="AC2" s="15" t="s">
+        <v>16</v>
       </c>
-      <c r="K2" s="14" t="s">
-        <v>49</v>
-      </c>
-      <c r="L2" s="14" t="s">
-        <v>50</v>
-      </c>
-      <c r="M2" s="14" t="s">
-        <v>51</v>
-      </c>
-      <c r="N2" s="14" t="s">
-        <v>52</v>
-      </c>
-      <c r="O2" s="14" t="s">
-        <v>32</v>
-      </c>
-      <c r="P2" s="15" t="s">
-        <v>53</v>
-      </c>
-      <c r="Q2" s="15" t="s">
-        <v>54</v>
-      </c>
-      <c r="R2" s="15" t="s">
-        <v>61</v>
-      </c>
-      <c r="S2" s="15" t="s">
-        <v>55</v>
-      </c>
-      <c r="T2" s="15" t="s">
-        <v>56</v>
-      </c>
-      <c r="U2" s="21" t="s">
-        <v>65</v>
-      </c>
-      <c r="V2" s="21" t="s">
-        <v>60</v>
-      </c>
-      <c r="W2" s="21" t="s">
-        <v>57</v>
-      </c>
-      <c r="X2" s="21" t="s">
-        <v>58</v>
-      </c>
-      <c r="Y2" s="21" t="s">
-        <v>59</v>
-      </c>
-      <c r="Z2" s="16" t="s">
+      <c r="AD2" s="16" t="s">
         <v>63</v>
       </c>
-      <c r="AA2" s="13" t="s">
-        <v>15</v>
-      </c>
-      <c r="AB2" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="AC2" s="15" t="s">
-        <v>17</v>
-      </c>
-      <c r="AD2" s="16" t="s">
-        <v>64</v>
-      </c>
       <c r="AE2" s="17" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="3" spans="1:31" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Added links to sites.
</commit_message>
<xml_diff>
--- a/The Blue Alliance/Templates/scouting_template.xlsx
+++ b/The Blue Alliance/Templates/scouting_template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/johnhurrell/Development/fairport-robotics/ScoutingPASSSync/The Blue Alliance/Templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1233944-BFF3-7F4C-BCD2-A35525035DA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A01C1E9-A94B-A14B-83B1-29F0442F27DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="MatchScoutingData" sheetId="1" r:id="rId1"/>
@@ -565,14 +565,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" textRotation="90"/>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" textRotation="90"/>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -592,14 +592,14 @@
     <xf numFmtId="0" fontId="1" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" textRotation="90"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -20890,7 +20890,7 @@
     <col min="1" max="1" width="16.5" customWidth="1"/>
     <col min="2" max="2" width="35" customWidth="1"/>
     <col min="3" max="3" width="50" customWidth="1"/>
-    <col min="4" max="6" width="12.83203125" style="22" customWidth="1"/>
+    <col min="4" max="6" width="20.83203125" style="22" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:29" ht="20" customHeight="1" x14ac:dyDescent="0.2">
@@ -20903,13 +20903,13 @@
       <c r="C1" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="D1" s="34" t="s">
+      <c r="D1" s="23" t="s">
         <v>77</v>
       </c>
-      <c r="E1" s="34" t="s">
+      <c r="E1" s="23" t="s">
         <v>78</v>
       </c>
-      <c r="F1" s="34" t="s">
+      <c r="F1" s="23" t="s">
         <v>79</v>
       </c>
       <c r="G1" s="5"/>
@@ -21168,14 +21168,14 @@
       <c r="R1" s="31"/>
       <c r="S1" s="31"/>
       <c r="T1" s="31"/>
-      <c r="U1" s="32" t="s">
+      <c r="U1" s="24" t="s">
         <v>63</v>
       </c>
-      <c r="V1" s="32"/>
-      <c r="W1" s="32"/>
-      <c r="X1" s="32"/>
-      <c r="Y1" s="32"/>
-      <c r="Z1" s="33"/>
+      <c r="V1" s="24"/>
+      <c r="W1" s="24"/>
+      <c r="X1" s="24"/>
+      <c r="Y1" s="24"/>
+      <c r="Z1" s="25"/>
     </row>
     <row r="2" spans="1:26" ht="130" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
@@ -29594,7 +29594,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:31" ht="17" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="24" t="s">
+      <c r="A1" s="33" t="s">
         <v>3</v>
       </c>
       <c r="B1" s="6"/>
@@ -29622,24 +29622,24 @@
       <c r="R1" s="31"/>
       <c r="S1" s="31"/>
       <c r="T1" s="31"/>
-      <c r="U1" s="32" t="s">
+      <c r="U1" s="24" t="s">
         <v>63</v>
       </c>
-      <c r="V1" s="32"/>
-      <c r="W1" s="32"/>
-      <c r="X1" s="32"/>
-      <c r="Y1" s="32"/>
-      <c r="Z1" s="32"/>
-      <c r="AA1" s="23" t="s">
+      <c r="V1" s="24"/>
+      <c r="W1" s="24"/>
+      <c r="X1" s="24"/>
+      <c r="Y1" s="24"/>
+      <c r="Z1" s="24"/>
+      <c r="AA1" s="32" t="s">
         <v>17</v>
       </c>
-      <c r="AB1" s="23"/>
-      <c r="AC1" s="23"/>
-      <c r="AD1" s="23"/>
-      <c r="AE1" s="23"/>
+      <c r="AB1" s="32"/>
+      <c r="AC1" s="32"/>
+      <c r="AD1" s="32"/>
+      <c r="AE1" s="32"/>
     </row>
     <row r="2" spans="1:31" ht="130" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="25"/>
+      <c r="A2" s="34"/>
       <c r="B2" s="12" t="s">
         <v>65</v>
       </c>

</xml_diff>

<commit_message>
Renamed to Team Summary.
</commit_message>
<xml_diff>
--- a/The Blue Alliance/Templates/scouting_template.xlsx
+++ b/The Blue Alliance/Templates/scouting_template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/johnhurrell/Development/fairport-robotics/ScoutingPASSSync/The Blue Alliance/Templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12834230-8E28-E34D-A3AE-D55E3252300F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5CE15DD-B325-0F4D-A707-2629B05A079C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18,15 +18,13 @@
     <sheet name="Teams" sheetId="3" r:id="rId3"/>
     <sheet name="Matches" sheetId="4" r:id="rId4"/>
     <sheet name="Team Scores" sheetId="5" r:id="rId5"/>
-    <sheet name="Team Summary Weightings" sheetId="12" r:id="rId6"/>
-    <sheet name="Team Summary" sheetId="9" r:id="rId7"/>
+    <sheet name="Team Summary" sheetId="12" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">Matches!$A$1:$H$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">MatchScoutingData!$A$1:$AA$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Team Scores'!$A$2:$AC$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Team Summary'!$A$2:$AC$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Team Summary Weightings'!$A$3:$AD$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Team Summary'!$A$3:$AD$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Teams!$A$1:$F$1</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -47,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2146" uniqueCount="592">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2112" uniqueCount="592">
   <si>
     <t>Key</t>
   </si>
@@ -1830,7 +1828,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="0.000"/>
+    <numFmt numFmtId="164" formatCode="0.000"/>
   </numFmts>
   <fonts count="9" x14ac:knownFonts="1">
     <font>
@@ -2113,7 +2111,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="69">
+  <cellXfs count="68">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -2189,25 +2187,49 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="1" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="1" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="1" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="8" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" textRotation="90"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2227,6 +2249,30 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -2251,57 +2297,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="3" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="1" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="1" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="1" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="1" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="7" fillId="8" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="1" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="1" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="1" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" textRotation="90"/>
-    </xf>
-    <xf numFmtId="165" fontId="1" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="3" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -54168,49 +54163,49 @@
   <dimension ref="A1:AC299"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="29" width="6.33203125" customWidth="1"/>
+    <col min="2" max="29" width="6.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:29" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A1" s="6"/>
       <c r="B1" s="6"/>
-      <c r="C1" s="47" t="s">
+      <c r="C1" s="63" t="s">
         <v>51</v>
       </c>
-      <c r="D1" s="48"/>
-      <c r="E1" s="48"/>
-      <c r="F1" s="49" t="s">
+      <c r="D1" s="64"/>
+      <c r="E1" s="64"/>
+      <c r="F1" s="65" t="s">
         <v>15</v>
       </c>
-      <c r="G1" s="50"/>
-      <c r="H1" s="50"/>
-      <c r="I1" s="50"/>
-      <c r="J1" s="50"/>
-      <c r="K1" s="50"/>
-      <c r="L1" s="50"/>
-      <c r="M1" s="50"/>
-      <c r="N1" s="50"/>
-      <c r="O1" s="51"/>
-      <c r="P1" s="41" t="s">
+      <c r="G1" s="66"/>
+      <c r="H1" s="66"/>
+      <c r="I1" s="66"/>
+      <c r="J1" s="66"/>
+      <c r="K1" s="66"/>
+      <c r="L1" s="66"/>
+      <c r="M1" s="66"/>
+      <c r="N1" s="66"/>
+      <c r="O1" s="67"/>
+      <c r="P1" s="49" t="s">
         <v>16</v>
       </c>
-      <c r="Q1" s="42"/>
-      <c r="R1" s="43"/>
-      <c r="S1" s="44" t="s">
+      <c r="Q1" s="50"/>
+      <c r="R1" s="51"/>
+      <c r="S1" s="60" t="s">
         <v>31</v>
       </c>
-      <c r="T1" s="45"/>
-      <c r="U1" s="45"/>
-      <c r="V1" s="45"/>
-      <c r="W1" s="45"/>
-      <c r="X1" s="46"/>
-      <c r="Y1" s="31" t="s">
+      <c r="T1" s="61"/>
+      <c r="U1" s="61"/>
+      <c r="V1" s="61"/>
+      <c r="W1" s="61"/>
+      <c r="X1" s="62"/>
+      <c r="Y1" s="53" t="s">
         <v>17</v>
       </c>
-      <c r="Z1" s="32"/>
-      <c r="AA1" s="32"/>
-      <c r="AB1" s="32"/>
-      <c r="AC1" s="33"/>
+      <c r="Z1" s="54"/>
+      <c r="AA1" s="54"/>
+      <c r="AB1" s="54"/>
+      <c r="AC1" s="55"/>
     </row>
     <row r="2" spans="1:29" ht="145" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
@@ -62041,138 +62036,138 @@
   <dimension ref="A1:AD32"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="30" width="6.33203125" customWidth="1"/>
+    <col min="2" max="30" width="6.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:30" ht="17" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="65" t="s">
+      <c r="A1" s="56" t="s">
         <v>590</v>
       </c>
-      <c r="B1" s="66"/>
-      <c r="C1" s="62"/>
-      <c r="D1" s="52" t="s">
+      <c r="B1" s="57"/>
+      <c r="C1" s="40"/>
+      <c r="D1" s="43" t="s">
         <v>51</v>
       </c>
-      <c r="E1" s="35"/>
-      <c r="F1" s="36"/>
-      <c r="G1" s="38" t="s">
+      <c r="E1" s="44"/>
+      <c r="F1" s="45"/>
+      <c r="G1" s="46" t="s">
         <v>15</v>
       </c>
-      <c r="H1" s="39"/>
-      <c r="I1" s="39"/>
-      <c r="J1" s="39"/>
-      <c r="K1" s="39"/>
-      <c r="L1" s="39"/>
-      <c r="M1" s="39"/>
-      <c r="N1" s="39"/>
-      <c r="O1" s="39"/>
-      <c r="P1" s="40"/>
-      <c r="Q1" s="41" t="s">
+      <c r="H1" s="47"/>
+      <c r="I1" s="47"/>
+      <c r="J1" s="47"/>
+      <c r="K1" s="47"/>
+      <c r="L1" s="47"/>
+      <c r="M1" s="47"/>
+      <c r="N1" s="47"/>
+      <c r="O1" s="47"/>
+      <c r="P1" s="48"/>
+      <c r="Q1" s="49" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="42"/>
-      <c r="S1" s="43"/>
-      <c r="T1" s="37" t="s">
+      <c r="R1" s="50"/>
+      <c r="S1" s="51"/>
+      <c r="T1" s="52" t="s">
         <v>31</v>
       </c>
-      <c r="U1" s="37"/>
-      <c r="V1" s="37"/>
-      <c r="W1" s="37"/>
-      <c r="X1" s="37"/>
-      <c r="Y1" s="37"/>
-      <c r="Z1" s="31" t="s">
+      <c r="U1" s="52"/>
+      <c r="V1" s="52"/>
+      <c r="W1" s="52"/>
+      <c r="X1" s="52"/>
+      <c r="Y1" s="52"/>
+      <c r="Z1" s="53" t="s">
         <v>17</v>
       </c>
-      <c r="AA1" s="32"/>
-      <c r="AB1" s="32"/>
-      <c r="AC1" s="32"/>
-      <c r="AD1" s="33"/>
+      <c r="AA1" s="54"/>
+      <c r="AB1" s="54"/>
+      <c r="AC1" s="54"/>
+      <c r="AD1" s="55"/>
     </row>
     <row r="2" spans="1:30" ht="17" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="67"/>
-      <c r="B2" s="68"/>
-      <c r="C2" s="64">
-        <v>1</v>
-      </c>
-      <c r="D2" s="63">
-        <v>1</v>
-      </c>
-      <c r="E2" s="53">
-        <v>1</v>
-      </c>
-      <c r="F2" s="53">
-        <v>1</v>
-      </c>
-      <c r="G2" s="54">
-        <v>1</v>
-      </c>
-      <c r="H2" s="55">
-        <v>1</v>
-      </c>
-      <c r="I2" s="55">
-        <v>1</v>
-      </c>
-      <c r="J2" s="55">
-        <v>1</v>
-      </c>
-      <c r="K2" s="55">
-        <v>1</v>
-      </c>
-      <c r="L2" s="55">
-        <v>1</v>
-      </c>
-      <c r="M2" s="55">
-        <v>1</v>
-      </c>
-      <c r="N2" s="55">
-        <v>1</v>
-      </c>
-      <c r="O2" s="55">
-        <v>1</v>
-      </c>
-      <c r="P2" s="55">
-        <v>1</v>
-      </c>
-      <c r="Q2" s="56">
-        <v>1</v>
-      </c>
-      <c r="R2" s="57">
-        <v>1</v>
-      </c>
-      <c r="S2" s="57">
-        <v>1</v>
-      </c>
-      <c r="T2" s="58">
-        <v>1</v>
-      </c>
-      <c r="U2" s="58">
-        <v>1</v>
-      </c>
-      <c r="V2" s="58">
-        <v>1</v>
-      </c>
-      <c r="W2" s="58">
-        <v>1</v>
-      </c>
-      <c r="X2" s="58">
-        <v>1</v>
-      </c>
-      <c r="Y2" s="58">
-        <v>1</v>
-      </c>
-      <c r="Z2" s="59">
-        <v>1</v>
-      </c>
-      <c r="AA2" s="60">
-        <v>1</v>
-      </c>
-      <c r="AB2" s="60">
-        <v>1</v>
-      </c>
-      <c r="AC2" s="60">
-        <v>1</v>
-      </c>
-      <c r="AD2" s="61">
+      <c r="A2" s="58"/>
+      <c r="B2" s="59"/>
+      <c r="C2" s="42">
+        <v>1</v>
+      </c>
+      <c r="D2" s="41">
+        <v>1</v>
+      </c>
+      <c r="E2" s="31">
+        <v>1</v>
+      </c>
+      <c r="F2" s="31">
+        <v>1</v>
+      </c>
+      <c r="G2" s="32">
+        <v>1</v>
+      </c>
+      <c r="H2" s="33">
+        <v>1</v>
+      </c>
+      <c r="I2" s="33">
+        <v>1</v>
+      </c>
+      <c r="J2" s="33">
+        <v>1</v>
+      </c>
+      <c r="K2" s="33">
+        <v>1</v>
+      </c>
+      <c r="L2" s="33">
+        <v>1</v>
+      </c>
+      <c r="M2" s="33">
+        <v>1</v>
+      </c>
+      <c r="N2" s="33">
+        <v>1</v>
+      </c>
+      <c r="O2" s="33">
+        <v>1</v>
+      </c>
+      <c r="P2" s="33">
+        <v>1</v>
+      </c>
+      <c r="Q2" s="34">
+        <v>1</v>
+      </c>
+      <c r="R2" s="35">
+        <v>1</v>
+      </c>
+      <c r="S2" s="35">
+        <v>1</v>
+      </c>
+      <c r="T2" s="36">
+        <v>1</v>
+      </c>
+      <c r="U2" s="36">
+        <v>1</v>
+      </c>
+      <c r="V2" s="36">
+        <v>1</v>
+      </c>
+      <c r="W2" s="36">
+        <v>1</v>
+      </c>
+      <c r="X2" s="36">
+        <v>1</v>
+      </c>
+      <c r="Y2" s="36">
+        <v>1</v>
+      </c>
+      <c r="Z2" s="37">
+        <v>1</v>
+      </c>
+      <c r="AA2" s="38">
+        <v>1</v>
+      </c>
+      <c r="AB2" s="38">
+        <v>1</v>
+      </c>
+      <c r="AC2" s="38">
+        <v>1</v>
+      </c>
+      <c r="AD2" s="39">
         <v>1</v>
       </c>
     </row>
@@ -62387,251 +62382,12 @@
   </sheetData>
   <autoFilter ref="A3:AD3" xr:uid="{8299AA4A-5D09-AD47-9627-5C6D2535B1BB}"/>
   <mergeCells count="6">
+    <mergeCell ref="A1:B2"/>
     <mergeCell ref="D1:F1"/>
     <mergeCell ref="G1:P1"/>
     <mergeCell ref="Q1:S1"/>
     <mergeCell ref="T1:Y1"/>
     <mergeCell ref="Z1:AD1"/>
-    <mergeCell ref="A1:B2"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8299AA4A-5D09-AD47-9627-5C6D2535B1BB}">
-  <dimension ref="A1:AC31"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="2" max="29" width="6.33203125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:29" ht="17" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="6"/>
-      <c r="B1" s="6"/>
-      <c r="C1" s="34" t="s">
-        <v>51</v>
-      </c>
-      <c r="D1" s="35"/>
-      <c r="E1" s="36"/>
-      <c r="F1" s="38" t="s">
-        <v>15</v>
-      </c>
-      <c r="G1" s="39"/>
-      <c r="H1" s="39"/>
-      <c r="I1" s="39"/>
-      <c r="J1" s="39"/>
-      <c r="K1" s="39"/>
-      <c r="L1" s="39"/>
-      <c r="M1" s="39"/>
-      <c r="N1" s="39"/>
-      <c r="O1" s="40"/>
-      <c r="P1" s="41" t="s">
-        <v>16</v>
-      </c>
-      <c r="Q1" s="42"/>
-      <c r="R1" s="43"/>
-      <c r="S1" s="37" t="s">
-        <v>31</v>
-      </c>
-      <c r="T1" s="37"/>
-      <c r="U1" s="37"/>
-      <c r="V1" s="37"/>
-      <c r="W1" s="37"/>
-      <c r="X1" s="37"/>
-      <c r="Y1" s="31" t="s">
-        <v>17</v>
-      </c>
-      <c r="Z1" s="32"/>
-      <c r="AA1" s="32"/>
-      <c r="AB1" s="32"/>
-      <c r="AC1" s="33"/>
-    </row>
-    <row r="2" spans="1:29" ht="145" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" s="24" t="s">
-        <v>32</v>
-      </c>
-      <c r="C2" s="18" t="s">
-        <v>47</v>
-      </c>
-      <c r="D2" s="19" t="s">
-        <v>19</v>
-      </c>
-      <c r="E2" s="19" t="s">
-        <v>20</v>
-      </c>
-      <c r="F2" s="20" t="s">
-        <v>21</v>
-      </c>
-      <c r="G2" s="21" t="s">
-        <v>22</v>
-      </c>
-      <c r="H2" s="21" t="s">
-        <v>48</v>
-      </c>
-      <c r="I2" s="21" t="s">
-        <v>588</v>
-      </c>
-      <c r="J2" s="21" t="s">
-        <v>589</v>
-      </c>
-      <c r="K2" s="21" t="s">
-        <v>23</v>
-      </c>
-      <c r="L2" s="21" t="s">
-        <v>24</v>
-      </c>
-      <c r="M2" s="21" t="s">
-        <v>49</v>
-      </c>
-      <c r="N2" s="21" t="s">
-        <v>50</v>
-      </c>
-      <c r="O2" s="21" t="s">
-        <v>25</v>
-      </c>
-      <c r="P2" s="22" t="s">
-        <v>26</v>
-      </c>
-      <c r="Q2" s="23" t="s">
-        <v>29</v>
-      </c>
-      <c r="R2" s="23" t="s">
-        <v>27</v>
-      </c>
-      <c r="S2" s="25" t="s">
-        <v>52</v>
-      </c>
-      <c r="T2" s="26" t="s">
-        <v>587</v>
-      </c>
-      <c r="U2" s="26" t="s">
-        <v>585</v>
-      </c>
-      <c r="V2" s="26" t="s">
-        <v>586</v>
-      </c>
-      <c r="W2" s="26" t="s">
-        <v>28</v>
-      </c>
-      <c r="X2" s="26" t="s">
-        <v>30</v>
-      </c>
-      <c r="Y2" s="24" t="s">
-        <v>14</v>
-      </c>
-      <c r="Z2" s="28" t="s">
-        <v>15</v>
-      </c>
-      <c r="AA2" s="28" t="s">
-        <v>16</v>
-      </c>
-      <c r="AB2" s="28" t="s">
-        <v>31</v>
-      </c>
-      <c r="AC2" s="29" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="3" spans="1:29" x14ac:dyDescent="0.2">
-      <c r="A3" s="30"/>
-    </row>
-    <row r="4" spans="1:29" x14ac:dyDescent="0.2">
-      <c r="A4" s="30"/>
-    </row>
-    <row r="5" spans="1:29" x14ac:dyDescent="0.2">
-      <c r="A5" s="30"/>
-    </row>
-    <row r="6" spans="1:29" x14ac:dyDescent="0.2">
-      <c r="A6" s="30"/>
-    </row>
-    <row r="7" spans="1:29" x14ac:dyDescent="0.2">
-      <c r="A7" s="30"/>
-    </row>
-    <row r="8" spans="1:29" x14ac:dyDescent="0.2">
-      <c r="A8" s="30"/>
-    </row>
-    <row r="9" spans="1:29" x14ac:dyDescent="0.2">
-      <c r="A9" s="30"/>
-    </row>
-    <row r="10" spans="1:29" x14ac:dyDescent="0.2">
-      <c r="A10" s="30"/>
-    </row>
-    <row r="11" spans="1:29" x14ac:dyDescent="0.2">
-      <c r="A11" s="30"/>
-    </row>
-    <row r="12" spans="1:29" x14ac:dyDescent="0.2">
-      <c r="A12" s="30"/>
-    </row>
-    <row r="13" spans="1:29" x14ac:dyDescent="0.2">
-      <c r="A13" s="30"/>
-    </row>
-    <row r="14" spans="1:29" x14ac:dyDescent="0.2">
-      <c r="A14" s="30"/>
-    </row>
-    <row r="15" spans="1:29" x14ac:dyDescent="0.2">
-      <c r="A15" s="30"/>
-    </row>
-    <row r="16" spans="1:29" x14ac:dyDescent="0.2">
-      <c r="A16" s="30"/>
-    </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A17" s="30"/>
-    </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A18" s="30"/>
-    </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A19" s="30"/>
-    </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A20" s="30"/>
-    </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A21" s="30"/>
-    </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A22" s="30"/>
-    </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A23" s="30"/>
-    </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A24" s="30"/>
-    </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A25" s="30"/>
-    </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A26" s="30"/>
-    </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A27" s="30"/>
-    </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A28" s="30"/>
-    </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A29" s="30"/>
-    </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A30" s="30"/>
-    </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A31" s="30"/>
-    </row>
-  </sheetData>
-  <autoFilter ref="A2:AC2" xr:uid="{8299AA4A-5D09-AD47-9627-5C6D2535B1BB}"/>
-  <mergeCells count="5">
-    <mergeCell ref="Y1:AC1"/>
-    <mergeCell ref="C1:E1"/>
-    <mergeCell ref="S1:X1"/>
-    <mergeCell ref="F1:O1"/>
-    <mergeCell ref="P1:R1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>

<commit_message>
More updates to the template.
</commit_message>
<xml_diff>
--- a/The Blue Alliance/Templates/scouting_template.xlsx
+++ b/The Blue Alliance/Templates/scouting_template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/johnhurrell/Development/fairport-robotics/ScoutingPASSSync/The Blue Alliance/Templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3414EB1D-2C80-9D4B-ABDC-08FF3DDB4A33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B9D8AA6-0B69-5F4B-BFE0-0827B0F4FC41}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="MatchScoutingData" sheetId="1" r:id="rId1"/>
@@ -73625,7 +73625,7 @@
       <c r="A2" s="68"/>
       <c r="B2" s="69"/>
       <c r="C2" s="39">
-        <v>1</v>
+        <v>0.1</v>
       </c>
       <c r="D2" s="38">
         <v>1</v>
@@ -73796,11 +73796,11 @@
       </c>
       <c r="B4" s="53">
         <f>IF(A4&lt;&gt;"",SUM(C4:AB4),"")</f>
-        <v>13.689999999999996</v>
+        <v>12.824199999999999</v>
       </c>
       <c r="C4" s="49">
         <f>IF($A4&lt;&gt;"",PERCENTRANK('Team Scores'!B$3:B$955, 'Team Scores'!B3, 3) * C$2, "")</f>
-        <v>0.96199999999999997</v>
+        <v>9.6200000000000008E-2</v>
       </c>
       <c r="D4" s="49">
         <f>IF($A4&lt;&gt;"",PERCENTRANK('Team Scores'!C$3:C$955, 'Team Scores'!C3, 3) * D$2, "")</f>
@@ -78014,11 +78014,11 @@
       </c>
       <c r="B41" s="53">
         <f>IF(A41&lt;&gt;"",SUM(C41:AB41),"")</f>
-        <v>16.894000000000002</v>
+        <v>16.028200000000002</v>
       </c>
       <c r="C41" s="49">
         <f>IF($A41&lt;&gt;"",PERCENTRANK('Team Scores'!B$3:B$955, 'Team Scores'!B40, 3) * C$2, "")</f>
-        <v>0.96199999999999997</v>
+        <v>9.6200000000000008E-2</v>
       </c>
       <c r="D41" s="49">
         <f>IF($A41&lt;&gt;"",PERCENTRANK('Team Scores'!C$3:C$955, 'Team Scores'!C40, 3) * D$2, "")</f>
@@ -79382,11 +79382,11 @@
       </c>
       <c r="B53" s="53">
         <f>IF(A53&lt;&gt;"",SUM(C53:AB53),"")</f>
-        <v>13.745999999999999</v>
+        <v>12.880199999999999</v>
       </c>
       <c r="C53" s="49">
         <f>IF($A53&lt;&gt;"",PERCENTRANK('Team Scores'!B$3:B$955, 'Team Scores'!B52, 3) * C$2, "")</f>
-        <v>0.96199999999999997</v>
+        <v>9.6200000000000008E-2</v>
       </c>
       <c r="D53" s="49">
         <f>IF($A53&lt;&gt;"",PERCENTRANK('Team Scores'!C$3:C$955, 'Team Scores'!C52, 3) * D$2, "")</f>

</xml_diff>